<commit_message>
feat: implement exam management module with dynamic form generation and backend integration for external faculty and university admin workflows
</commit_message>
<xml_diff>
--- a/mp-ems/login_data.xlsx
+++ b/mp-ems/login_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Intense\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MP_DHE_EMS_RD\mp-ems\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D87EFBB1-4DA8-4A32-8538-18395E6A898E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3043EA5-DAAE-44F9-9B3C-BC20CF5CD349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="43">
   <si>
     <t>Role</t>
   </si>
@@ -131,13 +131,31 @@
   </si>
   <si>
     <t>anil.kumar@abc.com</t>
+  </si>
+  <si>
+    <t>sgsits@ems.com</t>
+  </si>
+  <si>
+    <t>Admin@123</t>
+  </si>
+  <si>
+    <t>mp_college_admin@mpu.ac.in</t>
+  </si>
+  <si>
+    <t>mpadmin@2024</t>
+  </si>
+  <si>
+    <t>mp university college login</t>
+  </si>
+  <si>
+    <t>sgsit college login</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -165,6 +183,21 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -199,17 +232,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -510,7 +546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.5703125" customWidth="1"/>
@@ -520,294 +556,299 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="2"/>
     </row>
     <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="2"/>
     </row>
     <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="2"/>
+      <c r="C4" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="2"/>
+      <c r="C5" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="2"/>
+      <c r="C6" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="2"/>
+      <c r="C7" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="2"/>
+      <c r="C8" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="2"/>
+      <c r="C9" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="2"/>
+      <c r="C10" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="2"/>
+      <c r="C11" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="2"/>
+      <c r="C12" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="2"/>
+      <c r="C13" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="2"/>
+      <c r="C14" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="2"/>
+      <c r="C15" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="2"/>
-    </row>
-    <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="C16" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="2"/>
-    </row>
-    <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="C17" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="2"/>
-    </row>
-    <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="C18" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="C19" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="C20" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="2"/>
-    </row>
-    <row r="22" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="C21" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="2"/>
-    </row>
-    <row r="23" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+    </row>
+    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D23" s="2"/>
-    </row>
-    <row r="24" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+      <c r="C23" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="2"/>
+      <c r="C24" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B25" r:id="rId1" tooltip="mailto:sgsits@ems.com" display="mailto:sgsits@ems.com" xr:uid="{82BDD69D-EE14-4112-B41B-6ED4A32FC70F}"/>
+    <hyperlink ref="C25" r:id="rId2" xr:uid="{123CAABE-FE7C-4244-84A5-04392ABFCE21}"/>
+    <hyperlink ref="B26" r:id="rId3" tooltip="mailto:mp_college_admin@mpu.ac.in" display="mailto:mp_college_admin@mpu.ac.in" xr:uid="{7E1DE97D-DD71-4445-A444-299AE38C5127}"/>
+    <hyperlink ref="C26" r:id="rId4" tooltip="mailto:mpadmin@2024" display="mailto:mpadmin@2024" xr:uid="{31A5B18B-7167-4461-A8A4-BB36EF31D3A1}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>